<commit_message>
moved the nrl tab again to make it somewhat of a different app so you can switch between the nrl and nba tabs
</commit_message>
<xml_diff>
--- a/Documentation/SEN_Major_Project_Gantt_Chart.xlsx
+++ b/Documentation/SEN_Major_Project_Gantt_Chart.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -670,6 +670,19 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="9" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -687,19 +700,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="15" fontId="9" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -784,6 +784,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -980,95 +984,95 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25"/>
-      <c r="O1" s="25"/>
-      <c r="P1" s="25"/>
-      <c r="Q1" s="25"/>
-      <c r="R1" s="25"/>
-      <c r="S1" s="25"/>
-      <c r="T1" s="25"/>
-      <c r="U1" s="25"/>
-      <c r="V1" s="25"/>
-      <c r="W1" s="25"/>
-      <c r="X1" s="25"/>
-      <c r="Y1" s="25"/>
-      <c r="Z1" s="25"/>
-      <c r="AA1" s="25"/>
-      <c r="AB1" s="25"/>
-      <c r="AC1" s="25"/>
-      <c r="AD1" s="25"/>
-      <c r="AE1" s="25"/>
-      <c r="AF1" s="25"/>
-      <c r="AG1" s="25"/>
-      <c r="AH1" s="25"/>
-      <c r="AI1" s="25"/>
-      <c r="AJ1" s="25"/>
-      <c r="AK1" s="25"/>
-      <c r="AL1" s="25"/>
-      <c r="AM1" s="25"/>
-      <c r="AN1" s="25"/>
-      <c r="AO1" s="25"/>
-      <c r="AP1" s="25"/>
-      <c r="AQ1" s="25"/>
-      <c r="AR1" s="25"/>
-      <c r="AS1" s="25"/>
-      <c r="AT1" s="25"/>
-      <c r="AU1" s="25"/>
-      <c r="AV1" s="25"/>
-      <c r="AW1" s="25"/>
-      <c r="AX1" s="25"/>
-      <c r="AY1" s="25"/>
-      <c r="AZ1" s="25"/>
-      <c r="BA1" s="25"/>
-      <c r="BB1" s="25"/>
-      <c r="BC1" s="25"/>
-      <c r="BD1" s="25"/>
-      <c r="BE1" s="25"/>
-      <c r="BF1" s="25"/>
-      <c r="BG1" s="25"/>
-      <c r="BH1" s="25"/>
-      <c r="BI1" s="25"/>
-      <c r="BJ1" s="25"/>
-      <c r="BK1" s="25"/>
-      <c r="BL1" s="25"/>
-      <c r="BM1" s="25"/>
-      <c r="BN1" s="25"/>
-      <c r="BO1" s="25"/>
-      <c r="BP1" s="25"/>
-      <c r="BQ1" s="25"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+      <c r="N1" s="30"/>
+      <c r="O1" s="30"/>
+      <c r="P1" s="30"/>
+      <c r="Q1" s="30"/>
+      <c r="R1" s="30"/>
+      <c r="S1" s="30"/>
+      <c r="T1" s="30"/>
+      <c r="U1" s="30"/>
+      <c r="V1" s="30"/>
+      <c r="W1" s="30"/>
+      <c r="X1" s="30"/>
+      <c r="Y1" s="30"/>
+      <c r="Z1" s="30"/>
+      <c r="AA1" s="30"/>
+      <c r="AB1" s="30"/>
+      <c r="AC1" s="30"/>
+      <c r="AD1" s="30"/>
+      <c r="AE1" s="30"/>
+      <c r="AF1" s="30"/>
+      <c r="AG1" s="30"/>
+      <c r="AH1" s="30"/>
+      <c r="AI1" s="30"/>
+      <c r="AJ1" s="30"/>
+      <c r="AK1" s="30"/>
+      <c r="AL1" s="30"/>
+      <c r="AM1" s="30"/>
+      <c r="AN1" s="30"/>
+      <c r="AO1" s="30"/>
+      <c r="AP1" s="30"/>
+      <c r="AQ1" s="30"/>
+      <c r="AR1" s="30"/>
+      <c r="AS1" s="30"/>
+      <c r="AT1" s="30"/>
+      <c r="AU1" s="30"/>
+      <c r="AV1" s="30"/>
+      <c r="AW1" s="30"/>
+      <c r="AX1" s="30"/>
+      <c r="AY1" s="30"/>
+      <c r="AZ1" s="30"/>
+      <c r="BA1" s="30"/>
+      <c r="BB1" s="30"/>
+      <c r="BC1" s="30"/>
+      <c r="BD1" s="30"/>
+      <c r="BE1" s="30"/>
+      <c r="BF1" s="30"/>
+      <c r="BG1" s="30"/>
+      <c r="BH1" s="30"/>
+      <c r="BI1" s="30"/>
+      <c r="BJ1" s="30"/>
+      <c r="BK1" s="30"/>
+      <c r="BL1" s="30"/>
+      <c r="BM1" s="30"/>
+      <c r="BN1" s="30"/>
+      <c r="BO1" s="30"/>
+      <c r="BP1" s="30"/>
+      <c r="BQ1" s="30"/>
     </row>
     <row r="2" spans="1:69" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="27" t="s">
+      <c r="B2" s="31"/>
+      <c r="C2" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="27"/>
-      <c r="E2" s="28" t="s">
+      <c r="D2" s="32"/>
+      <c r="E2" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="28"/>
-      <c r="G2" s="29" t="s">
+      <c r="F2" s="33"/>
+      <c r="G2" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="29"/>
+      <c r="H2" s="34"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -1141,71 +1145,71 @@
       <c r="G3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="24" t="s">
+      <c r="H3" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
-      <c r="M3" s="24"/>
-      <c r="N3" s="24"/>
-      <c r="O3" s="24"/>
-      <c r="P3" s="24"/>
-      <c r="Q3" s="24"/>
-      <c r="R3" s="24"/>
-      <c r="S3" s="24"/>
-      <c r="T3" s="24"/>
-      <c r="U3" s="24"/>
-      <c r="V3" s="24"/>
-      <c r="W3" s="24"/>
-      <c r="X3" s="24"/>
-      <c r="Y3" s="24"/>
-      <c r="Z3" s="24"/>
-      <c r="AA3" s="24"/>
-      <c r="AB3" s="24"/>
-      <c r="AC3" s="24"/>
-      <c r="AD3" s="24"/>
-      <c r="AE3" s="24"/>
-      <c r="AF3" s="24"/>
-      <c r="AG3" s="24"/>
-      <c r="AH3" s="24"/>
-      <c r="AI3" s="24"/>
-      <c r="AJ3" s="24"/>
-      <c r="AK3" s="24"/>
-      <c r="AL3" s="24"/>
-      <c r="AM3" s="24" t="s">
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="29"/>
+      <c r="N3" s="29"/>
+      <c r="O3" s="29"/>
+      <c r="P3" s="29"/>
+      <c r="Q3" s="29"/>
+      <c r="R3" s="29"/>
+      <c r="S3" s="29"/>
+      <c r="T3" s="29"/>
+      <c r="U3" s="29"/>
+      <c r="V3" s="29"/>
+      <c r="W3" s="29"/>
+      <c r="X3" s="29"/>
+      <c r="Y3" s="29"/>
+      <c r="Z3" s="29"/>
+      <c r="AA3" s="29"/>
+      <c r="AB3" s="29"/>
+      <c r="AC3" s="29"/>
+      <c r="AD3" s="29"/>
+      <c r="AE3" s="29"/>
+      <c r="AF3" s="29"/>
+      <c r="AG3" s="29"/>
+      <c r="AH3" s="29"/>
+      <c r="AI3" s="29"/>
+      <c r="AJ3" s="29"/>
+      <c r="AK3" s="29"/>
+      <c r="AL3" s="29"/>
+      <c r="AM3" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="AN3" s="24"/>
-      <c r="AO3" s="24"/>
-      <c r="AP3" s="24"/>
-      <c r="AQ3" s="24"/>
-      <c r="AR3" s="24"/>
-      <c r="AS3" s="24"/>
-      <c r="AT3" s="24"/>
-      <c r="AU3" s="24"/>
-      <c r="AV3" s="24"/>
-      <c r="AW3" s="24"/>
-      <c r="AX3" s="24"/>
-      <c r="AY3" s="24"/>
-      <c r="AZ3" s="24"/>
-      <c r="BA3" s="24"/>
-      <c r="BB3" s="24"/>
-      <c r="BC3" s="24"/>
-      <c r="BD3" s="24"/>
-      <c r="BE3" s="24"/>
-      <c r="BF3" s="24"/>
-      <c r="BG3" s="24"/>
-      <c r="BH3" s="24"/>
-      <c r="BI3" s="24"/>
-      <c r="BJ3" s="24"/>
-      <c r="BK3" s="24"/>
-      <c r="BL3" s="24"/>
-      <c r="BM3" s="24"/>
-      <c r="BN3" s="24"/>
-      <c r="BO3" s="24"/>
-      <c r="BP3" s="24"/>
+      <c r="AN3" s="29"/>
+      <c r="AO3" s="29"/>
+      <c r="AP3" s="29"/>
+      <c r="AQ3" s="29"/>
+      <c r="AR3" s="29"/>
+      <c r="AS3" s="29"/>
+      <c r="AT3" s="29"/>
+      <c r="AU3" s="29"/>
+      <c r="AV3" s="29"/>
+      <c r="AW3" s="29"/>
+      <c r="AX3" s="29"/>
+      <c r="AY3" s="29"/>
+      <c r="AZ3" s="29"/>
+      <c r="BA3" s="29"/>
+      <c r="BB3" s="29"/>
+      <c r="BC3" s="29"/>
+      <c r="BD3" s="29"/>
+      <c r="BE3" s="29"/>
+      <c r="BF3" s="29"/>
+      <c r="BG3" s="29"/>
+      <c r="BH3" s="29"/>
+      <c r="BI3" s="29"/>
+      <c r="BJ3" s="29"/>
+      <c r="BK3" s="29"/>
+      <c r="BL3" s="29"/>
+      <c r="BM3" s="29"/>
+      <c r="BN3" s="29"/>
+      <c r="BO3" s="29"/>
+      <c r="BP3" s="29"/>
       <c r="BQ3" s="3" t="s">
         <v>8</v>
       </c>
@@ -2480,7 +2484,7 @@
     </row>
     <row r="18" spans="1:69" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="13"/>
-      <c r="B18" s="33" t="s">
+      <c r="B18" s="27" t="s">
         <v>128</v>
       </c>
       <c r="C18" s="15" t="s">
@@ -2810,7 +2814,7 @@
       <c r="C22" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="D22" s="34"/>
+      <c r="D22" s="28"/>
       <c r="E22" s="20" t="s">
         <v>53</v>
       </c>
@@ -2888,7 +2892,7 @@
       </c>
       <c r="C23" s="8"/>
       <c r="D23" s="8"/>
-      <c r="E23" s="32" t="s">
+      <c r="E23" s="26" t="s">
         <v>58</v>
       </c>
       <c r="F23" s="8" t="s">
@@ -3277,7 +3281,7 @@
       </c>
       <c r="C28" s="15"/>
       <c r="D28" s="15"/>
-      <c r="E28" s="30" t="s">
+      <c r="E28" s="24" t="s">
         <v>58</v>
       </c>
       <c r="F28" s="15" t="s">
@@ -3328,15 +3332,15 @@
       <c r="AW28" s="17"/>
       <c r="AX28" s="17"/>
       <c r="AY28" s="17"/>
-      <c r="AZ28" s="31"/>
-      <c r="BA28" s="31"/>
-      <c r="BB28" s="31"/>
-      <c r="BC28" s="31"/>
-      <c r="BD28" s="31"/>
-      <c r="BE28" s="31"/>
-      <c r="BF28" s="31"/>
-      <c r="BG28" s="31"/>
-      <c r="BH28" s="31"/>
+      <c r="AZ28" s="25"/>
+      <c r="BA28" s="25"/>
+      <c r="BB28" s="25"/>
+      <c r="BC28" s="25"/>
+      <c r="BD28" s="25"/>
+      <c r="BE28" s="25"/>
+      <c r="BF28" s="25"/>
+      <c r="BG28" s="25"/>
+      <c r="BH28" s="25"/>
       <c r="BI28" s="17"/>
       <c r="BJ28" s="17"/>
       <c r="BK28" s="17"/>
@@ -3922,95 +3926,95 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25"/>
-      <c r="O1" s="25"/>
-      <c r="P1" s="25"/>
-      <c r="Q1" s="25"/>
-      <c r="R1" s="25"/>
-      <c r="S1" s="25"/>
-      <c r="T1" s="25"/>
-      <c r="U1" s="25"/>
-      <c r="V1" s="25"/>
-      <c r="W1" s="25"/>
-      <c r="X1" s="25"/>
-      <c r="Y1" s="25"/>
-      <c r="Z1" s="25"/>
-      <c r="AA1" s="25"/>
-      <c r="AB1" s="25"/>
-      <c r="AC1" s="25"/>
-      <c r="AD1" s="25"/>
-      <c r="AE1" s="25"/>
-      <c r="AF1" s="25"/>
-      <c r="AG1" s="25"/>
-      <c r="AH1" s="25"/>
-      <c r="AI1" s="25"/>
-      <c r="AJ1" s="25"/>
-      <c r="AK1" s="25"/>
-      <c r="AL1" s="25"/>
-      <c r="AM1" s="25"/>
-      <c r="AN1" s="25"/>
-      <c r="AO1" s="25"/>
-      <c r="AP1" s="25"/>
-      <c r="AQ1" s="25"/>
-      <c r="AR1" s="25"/>
-      <c r="AS1" s="25"/>
-      <c r="AT1" s="25"/>
-      <c r="AU1" s="25"/>
-      <c r="AV1" s="25"/>
-      <c r="AW1" s="25"/>
-      <c r="AX1" s="25"/>
-      <c r="AY1" s="25"/>
-      <c r="AZ1" s="25"/>
-      <c r="BA1" s="25"/>
-      <c r="BB1" s="25"/>
-      <c r="BC1" s="25"/>
-      <c r="BD1" s="25"/>
-      <c r="BE1" s="25"/>
-      <c r="BF1" s="25"/>
-      <c r="BG1" s="25"/>
-      <c r="BH1" s="25"/>
-      <c r="BI1" s="25"/>
-      <c r="BJ1" s="25"/>
-      <c r="BK1" s="25"/>
-      <c r="BL1" s="25"/>
-      <c r="BM1" s="25"/>
-      <c r="BN1" s="25"/>
-      <c r="BO1" s="25"/>
-      <c r="BP1" s="25"/>
-      <c r="BQ1" s="25"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+      <c r="N1" s="30"/>
+      <c r="O1" s="30"/>
+      <c r="P1" s="30"/>
+      <c r="Q1" s="30"/>
+      <c r="R1" s="30"/>
+      <c r="S1" s="30"/>
+      <c r="T1" s="30"/>
+      <c r="U1" s="30"/>
+      <c r="V1" s="30"/>
+      <c r="W1" s="30"/>
+      <c r="X1" s="30"/>
+      <c r="Y1" s="30"/>
+      <c r="Z1" s="30"/>
+      <c r="AA1" s="30"/>
+      <c r="AB1" s="30"/>
+      <c r="AC1" s="30"/>
+      <c r="AD1" s="30"/>
+      <c r="AE1" s="30"/>
+      <c r="AF1" s="30"/>
+      <c r="AG1" s="30"/>
+      <c r="AH1" s="30"/>
+      <c r="AI1" s="30"/>
+      <c r="AJ1" s="30"/>
+      <c r="AK1" s="30"/>
+      <c r="AL1" s="30"/>
+      <c r="AM1" s="30"/>
+      <c r="AN1" s="30"/>
+      <c r="AO1" s="30"/>
+      <c r="AP1" s="30"/>
+      <c r="AQ1" s="30"/>
+      <c r="AR1" s="30"/>
+      <c r="AS1" s="30"/>
+      <c r="AT1" s="30"/>
+      <c r="AU1" s="30"/>
+      <c r="AV1" s="30"/>
+      <c r="AW1" s="30"/>
+      <c r="AX1" s="30"/>
+      <c r="AY1" s="30"/>
+      <c r="AZ1" s="30"/>
+      <c r="BA1" s="30"/>
+      <c r="BB1" s="30"/>
+      <c r="BC1" s="30"/>
+      <c r="BD1" s="30"/>
+      <c r="BE1" s="30"/>
+      <c r="BF1" s="30"/>
+      <c r="BG1" s="30"/>
+      <c r="BH1" s="30"/>
+      <c r="BI1" s="30"/>
+      <c r="BJ1" s="30"/>
+      <c r="BK1" s="30"/>
+      <c r="BL1" s="30"/>
+      <c r="BM1" s="30"/>
+      <c r="BN1" s="30"/>
+      <c r="BO1" s="30"/>
+      <c r="BP1" s="30"/>
+      <c r="BQ1" s="30"/>
     </row>
     <row r="2" spans="1:69" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="27" t="s">
+      <c r="B2" s="31"/>
+      <c r="C2" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="27"/>
-      <c r="E2" s="28" t="s">
+      <c r="D2" s="32"/>
+      <c r="E2" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="28"/>
-      <c r="G2" s="29" t="s">
+      <c r="F2" s="33"/>
+      <c r="G2" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="29"/>
+      <c r="H2" s="34"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -4083,71 +4087,71 @@
       <c r="G3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="24" t="s">
+      <c r="H3" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
-      <c r="M3" s="24"/>
-      <c r="N3" s="24"/>
-      <c r="O3" s="24"/>
-      <c r="P3" s="24"/>
-      <c r="Q3" s="24"/>
-      <c r="R3" s="24"/>
-      <c r="S3" s="24"/>
-      <c r="T3" s="24"/>
-      <c r="U3" s="24"/>
-      <c r="V3" s="24"/>
-      <c r="W3" s="24"/>
-      <c r="X3" s="24"/>
-      <c r="Y3" s="24"/>
-      <c r="Z3" s="24"/>
-      <c r="AA3" s="24"/>
-      <c r="AB3" s="24"/>
-      <c r="AC3" s="24"/>
-      <c r="AD3" s="24"/>
-      <c r="AE3" s="24"/>
-      <c r="AF3" s="24"/>
-      <c r="AG3" s="24"/>
-      <c r="AH3" s="24"/>
-      <c r="AI3" s="24"/>
-      <c r="AJ3" s="24"/>
-      <c r="AK3" s="24"/>
-      <c r="AL3" s="24"/>
-      <c r="AM3" s="24" t="s">
+      <c r="I3" s="29"/>
+      <c r="J3" s="29"/>
+      <c r="K3" s="29"/>
+      <c r="L3" s="29"/>
+      <c r="M3" s="29"/>
+      <c r="N3" s="29"/>
+      <c r="O3" s="29"/>
+      <c r="P3" s="29"/>
+      <c r="Q3" s="29"/>
+      <c r="R3" s="29"/>
+      <c r="S3" s="29"/>
+      <c r="T3" s="29"/>
+      <c r="U3" s="29"/>
+      <c r="V3" s="29"/>
+      <c r="W3" s="29"/>
+      <c r="X3" s="29"/>
+      <c r="Y3" s="29"/>
+      <c r="Z3" s="29"/>
+      <c r="AA3" s="29"/>
+      <c r="AB3" s="29"/>
+      <c r="AC3" s="29"/>
+      <c r="AD3" s="29"/>
+      <c r="AE3" s="29"/>
+      <c r="AF3" s="29"/>
+      <c r="AG3" s="29"/>
+      <c r="AH3" s="29"/>
+      <c r="AI3" s="29"/>
+      <c r="AJ3" s="29"/>
+      <c r="AK3" s="29"/>
+      <c r="AL3" s="29"/>
+      <c r="AM3" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="AN3" s="24"/>
-      <c r="AO3" s="24"/>
-      <c r="AP3" s="24"/>
-      <c r="AQ3" s="24"/>
-      <c r="AR3" s="24"/>
-      <c r="AS3" s="24"/>
-      <c r="AT3" s="24"/>
-      <c r="AU3" s="24"/>
-      <c r="AV3" s="24"/>
-      <c r="AW3" s="24"/>
-      <c r="AX3" s="24"/>
-      <c r="AY3" s="24"/>
-      <c r="AZ3" s="24"/>
-      <c r="BA3" s="24"/>
-      <c r="BB3" s="24"/>
-      <c r="BC3" s="24"/>
-      <c r="BD3" s="24"/>
-      <c r="BE3" s="24"/>
-      <c r="BF3" s="24"/>
-      <c r="BG3" s="24"/>
-      <c r="BH3" s="24"/>
-      <c r="BI3" s="24"/>
-      <c r="BJ3" s="24"/>
-      <c r="BK3" s="24"/>
-      <c r="BL3" s="24"/>
-      <c r="BM3" s="24"/>
-      <c r="BN3" s="24"/>
-      <c r="BO3" s="24"/>
-      <c r="BP3" s="24"/>
+      <c r="AN3" s="29"/>
+      <c r="AO3" s="29"/>
+      <c r="AP3" s="29"/>
+      <c r="AQ3" s="29"/>
+      <c r="AR3" s="29"/>
+      <c r="AS3" s="29"/>
+      <c r="AT3" s="29"/>
+      <c r="AU3" s="29"/>
+      <c r="AV3" s="29"/>
+      <c r="AW3" s="29"/>
+      <c r="AX3" s="29"/>
+      <c r="AY3" s="29"/>
+      <c r="AZ3" s="29"/>
+      <c r="BA3" s="29"/>
+      <c r="BB3" s="29"/>
+      <c r="BC3" s="29"/>
+      <c r="BD3" s="29"/>
+      <c r="BE3" s="29"/>
+      <c r="BF3" s="29"/>
+      <c r="BG3" s="29"/>
+      <c r="BH3" s="29"/>
+      <c r="BI3" s="29"/>
+      <c r="BJ3" s="29"/>
+      <c r="BK3" s="29"/>
+      <c r="BL3" s="29"/>
+      <c r="BM3" s="29"/>
+      <c r="BN3" s="29"/>
+      <c r="BO3" s="29"/>
+      <c r="BP3" s="29"/>
       <c r="BQ3" s="3" t="s">
         <v>8</v>
       </c>

</xml_diff>